<commit_message>
Track 2: evidence triangulation, pre-registered validation, PEX5 call quality
</commit_message>
<xml_diff>
--- a/track2/pari25mib10005_track2_methods.xlsx
+++ b/track2/pari25mib10005_track2_methods.xlsx
@@ -724,7 +724,7 @@
 3) Convergence: all three routes agree that the checkpoint core cannot be drugged directly in the helpful direction, so an indirect BUBR1-stabilising strategy was chosen from the literature: NAD+ repletion (NAD+ -&gt; SIRT2 deacetylates BUBR1 K668 -&gt; less degradation; North et al. 2014).
 4) Candidates and tiers: niacin (approved medication; raised blood NAD+ up to 8-fold in humans) and nicotinamide riboside (paediatric safety data); backups NMN, nicotinamide; NAC and senolytics low-tier/reserve.
 5) Personalisation (local tools on the patient VCF): NAD+-conversion genes intact (both drugs usable); pharmacogenomics (CEP72, CYP3A5 vincristine-neuropathy risk; CYP2C19 intermediate); Factor V Leiden (family history); genome-wide inheritance-aware scan of genes for the unexplained features (possible second diagnosis PEX5, testable by a blood test).
-6) Validation plan: patient cells (BUBR1, K668 acetylation, missegregation; SIRT2-dependence), BubR1 hypomorphic mice, then a supervised n-of-1 only with clinicians and ethics oversight.</t>
+6) Pre-registered validation plan (explicit success/failure thresholds): patient cells (BUBR1, K668 acetylation, missegregation; SIRT2-dependence), BubR1 hypomorphic mice, then a supervised n-of-1 only with clinicians and ethics oversight.</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Mechanism: MVA genetics and BUBR1 biology (Hanks 2004; Suijkerbuijk 2010, 2012; Elowe 2011; Baker 2004); the NAD+ -&gt; SIRT2 -&gt; BubR1 lever (North 2014). Candidates: paediatric NR safety (Veenhuis 2021; Presterud 2024; Neuropediatrics 2023 case), niacin NAD+ repletion in humans (Pirinen 2020), senolytic and antioxidant evidence (Baker 2011; Matsuda 2016). Curation: evidence tiers (A/B/C), a documented hazard list of drug classes never to propose, curated mechanisms for research compounds the databases do not annotate, and clinician notes. Every reference was checked against PubMed or the publisher; two claims were corrected during review (a senolytic study used genetic, not drug, clearance; NR is patent-protected, not off-patent).</t>
+          <t>Mechanism: MVA genetics and BUBR1 biology (Hanks 2004; Suijkerbuijk 2010, 2012; Elowe 2011; Baker 2004); the NAD+ -&gt; SIRT2 -&gt; BubR1 lever (North 2014), with independent support from SIRT2 genetics (Kim 2011: SIRT2 loss causes aneuploidy and tumours). Candidates: paediatric NR safety (Veenhuis 2021; Presterud 2024; Neuropediatrics 2023 case), niacin NAD+ repletion in humans (Pirinen 2020), a randomised placebo-controlled NR trial in Werner syndrome (Shoji 2025), senolytic and antioxidant evidence (Baker 2011; Matsuda 2016). Curation: evidence tiers (A/B/C), a documented hazard list of drug classes never to propose, curated mechanisms for research compounds the databases do not annotate, and clinician notes. Every reference was checked against PubMed or the publisher; two claims were corrected during review (a senolytic study used genetic, not drug, clearance; NR is patent-protected, not off-patent).</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
           <t>We characterised a compound-heterozygous BUB1B genotype as a loss-of-function hypomorph: a truncating allele predicted to undergo nonsense-mediated decay (LOFTEE high-confidence) and a kinase-domain missense allele predicted to destabilise the protein (AlphaMissense 0.92, no splice effect). The therapeutic goal is therefore to stabilise residual BUBR1 without weakening the spindle assembly checkpoint or adding cancer risk.
 Candidates were sought through three independent, scripted routes. A gene-first screen queried DGIdb and Open Targets across BUB1B, direction-annotated modifiers and STRING partners (552 records), applying layered safety filters (mitotic and genotoxic classes, all WHO ATC L01 antineoplastics, wrong-direction agents, a whole-drug mechanism check). A phenotype-first analysis scored all HPO genes against the patient's features, recovered BUB1B (16th of 2,479), identified a checkpoint module (KEGG cell cycle FDR 5.9e-10) and tested each feature for links to BUB1B's network. A transcriptome-first route compared the LINCS BUB1B knockout signature with 5,425 compounds, testing a pre-specified NAD+/sirtuin hypothesis. All three routes agree that the checkpoint core cannot be safely drugged directly. The lead is therefore NAD+ repletion, acting through SIRT2-mediated deacetylation of BUBR1 (shown to raise BubR1 in mice): niacin, an approved medicine that raised blood NAD+ up to 8-fold in humans, or nicotinamide riboside, which has open-label safety data in children. Local checks of the patient's genome show both drugs' NAD+ conversion pathways are intact, flag two vincristine-neuropathy risk genotypes and Factor V Leiden, and an inheritance-aware genome-wide scan raises one testable second-diagnosis candidate (PEX5) for features not explained by MVA.
 Strengths: mechanism supported by standard variant-effect predictors; three independent routes with explicit convergence; a pre-specified test reported honestly; safety-first filtering that removed several hazardous agents missed by single-source annotation; a methodological finding that naive signature reversal favours drugs silencing the p53/interferon alarm (93 of the top 100), unsafe in chromosome-instability disorders; personalised, clinically actionable checks; gene-agnostic tools that run with one command each and were tested on TRIP13 and CEP57.
-Limitations: the lead rests mainly on one mouse study; the pre-specified transcriptomic test was not significant (p = 0.085), and transcripts cannot capture protein-stability effects; nothing is validated experimentally; NR safety data come from another disease; database results drift between runs; the genome scans cover small coding variants only (no structural variants or phasing). All proposals are hypotheses for investigation, not treatment advice.</t>
+Limitations: direct evidence that NAD+ raises BUBR1 is from mice (human evidence covers NAD+ raising and safety, including a randomised trial in Werner syndrome), so a pre-registered cell experiment with explicit success and failure thresholds comes first; the pre-specified transcriptomic test was not significant (p = 0.085), and transcripts cannot capture protein-stability effects; nothing is validated experimentally; NR safety data come from another disease; database results drift between runs; the genome scans cover small coding variants only (no structural variants or phasing). All proposals are hypotheses for investigation, not treatment advice.</t>
         </is>
       </c>
     </row>

</xml_diff>